<commit_message>
Split the monolithic design doc into four focused guides for easier navigation.
Add water supply and drip irrigation (installation doc §2.6), refresh cross-references in AGENTS/README, and regenerate the BOM from updated doc paths.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/smart-greenhouse-bom.xlsx
+++ b/docs/smart-greenhouse-bom.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Рекомендуемый хост HA; док. §1.1; оригинальная плата</t>
+          <t>Рекомендуемый хост HA; док. 02 §1.1; оригинальная плата</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PoE + слот NVMe; док. §1.1; оригинал Waveshare</t>
+          <t>PoE + слот NVMe; док. 02 §1.1; оригинал Waveshare</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Загрузочный диск для HA OS; док. §1.1; форм‑фактор 2230 редкий — проверить 2230 перед покупкой (не 2280)</t>
+          <t>Загрузочный диск для HA OS; док. 02 §1.1; форм‑фактор 2230 редкий — проверить 2230 перед покупкой (не 2280)</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Охлаждение в сетевом шкафу; док. §1.1; официальный Active Cooler (~841 ₽) + алюминиевый корпус (~859 ₽, onpad.ru)</t>
+          <t>Охлаждение в сетевом шкафу; док. 02 §1.1; официальный Active Cooler (~841 ₽) + алюминиевый корпус (~859 ₽, onpad.ru)</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; Pi HA к PoE‑коммутатору; док. §1.1 — кол‑во 0 к заказу</t>
+          <t>Уже есть; Pi HA к PoE‑коммутатору; док. 02 §1.1 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; док. §1.2 — кол‑во 0 к заказу</t>
+          <t>Уже есть; док. 02 §1.2 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; наружная PoE AP ~5 м от теплицы; док. §1.2/§3</t>
+          <t>Уже есть; наружная PoE AP ~5 м от теплицы; док. 02 §1.2/01 §3</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; питает Pi HA + Stellar 6; док. §1.2</t>
+          <t>Уже есть; питает Pi HA + Stellar 6; док. 02 §1.2</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; ~15–20 м наружный Cat6 к mesh AP; док. §1.2/§3 — кол‑во 0 к заказу</t>
+          <t>Уже есть; ~15–20 м наружный Cat6 к mesh AP; док. 02 §1.2/01 §3 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>greenhouse-watering + greenhouse-climate; док. §1.3; разъём U.FL для внешней антенны</t>
+          <t>greenhouse-watering + greenhouse-climate; док. 04 §1.3; разъём U.FL для внешней антенны</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Внешние антенны вне металлического корпуса; док. §1.3; реселлер AliExpress — доставка 2–4 нед. vs местный склад</t>
+          <t>Внешние антенны вне металлического корпуса; док. 04 §1.3; реселлер AliExpress — доставка 2–4 нед. vs местный склад</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Питание логики: ESP32, датчики, PCA9685 VCC; док. §1.3/§2.5; оригинал Mean Well</t>
+          <t>Питание логики: ESP32, датчики, PCA9685 VCC; док. 04 §1.3/04 §2.5; оригинал Mean Well</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Питание реле и соленоидов; док. §1.3/§2.5; оригинал Mean Well</t>
+          <t>Питание реле и соленоидов; док. 04 §1.3/04 §2.5; оригинал Mean Well</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>По одному на ESP32 полива (клапаны полива и бака); док. §1.3/§1.5; SRD-12VDC-SL-C + PC817</t>
+          <t>По одному на ESP32 полива (клапаны полива и бака); док. 04 §1.3/03 §1.5; SRD-12VDC-SL-C + PC817</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Драйвер MG996R на greenhouse-climate; док. §1.3/§2.4</t>
+          <t>Драйвер MG996R на greenhouse-climate; док. 04 §1.3/04 §2.4</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Уже в наличии по док.; по одному на катушку реле/соленоида; док. §2.1</t>
+          <t>Уже в наличии по док.; по одному на катушку реле/соленоида; док. 04 §2.1</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Полевой щит у теплицы; док. §1.3; DKC R5ST0342 с монтажной платой</t>
+          <t>Полевой щит у теплицы; док. 04 §1.3; DKC R5ST0342 с монтажной платой</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>1 комплект; WAGO 221 + сальники DKC PG + DIN‑рейка; док. §1.3; оценка набора</t>
+          <t>1 комплект; WAGO 221 + сальники DKC PG + DIN‑рейка; док. 04 §1.3; оценка набора</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Линии датчиков внутрь теплицы; док. §1.3/§2.5; Extralink EX.32341 или аналог DKC outdoor FTP</t>
+          <t>Линии датчиков внутрь теплицы; док. 04 §1.3/04 §2.5; Extralink EX.32341 или аналог DKC outdoor FTP</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Опционально; удерживает клапаны в безопасном состоянии при отключении питания; док. §1.3/§6.4; класс WGP V1203</t>
+          <t>Опционально; удерживает клапаны в безопасном состоянии при отключении питания; док. 04 §1.3/01 §6.4; класс WGP V1203</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Антиконденсат в корпусе; док. §1.3/§5.1; вентиляционный винт IP67 (аналог Gore vent)</t>
+          <t>Антиконденсат в корпусе; док. 04 §1.3/01 §5.1; вентиляционный винт IP67 (аналог Gore vent)</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Оценка; док. §2.5/§6.4; IEK/DEK 1P 10 A</t>
+          <t>Оценка; док. 04 §2.5/01 §6.4; IEK/DEK 1P 10 A</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Отдельно от LRS-50-5; док. §2.4/§5.2; закрытый БП DONE 5 V 3 A 15 W</t>
+          <t>Отдельно от LRS-50-5; док. 04 §2.4/01 §5.2; закрытый БП DONE 5 V 3 A 15 W</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; подтяжки DS18B20 + I2C; док. §2.1 — кол‑во 0 к заказу</t>
+          <t>Уже есть; подтяжки DS18B20 + I2C; док. 04 §2.1 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; опциональный debounce поплавка; док. §5.2 — кол‑во 0 к заказу</t>
+          <t>Уже есть; опциональный debounce поплавка; док. 01 §5.2 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Центр, север, юг; I2C; док. §1.4/§2.3</t>
+          <t>Центр, север, юг; I2C; док. 03 §1.4 / 04 §2.3</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Потолок + уровень растений; док. §1.4</t>
+          <t>Потолок + уровень растений; док. 03 §1.4</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Бак + линия полива; OneWire; док. §1.4/§2.2</t>
+          <t>Бак + линия полива; OneWire; док. 03 §1.4 / 04 §2.2</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Верхний уровень бака; док. §1.4/§2.2; бытовой поплавок (не промышленный ПДУ)</t>
+          <t>Верхний уровень бака; док. 03 §1.4 / 04 §2.2; бытовой поплавок (не промышленный ПДУ)</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Учёт полива и наполнения бака; док. §1.4</t>
+          <t>Учёт полива и наполнения бака; док. 03 §1.4</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Полив + наполнение бака; fail-safe NC; док. §1.5; латунь 12 V DC прямого действия; реселлер AliExpress — проверить NC и мин. давление 0 bar</t>
+          <t>Полив + наполнение бака; fail-safe NC; док. 03 §1.5; латунь 12 V DC прямого действия; реселлер AliExpress — проверить NC и мин. давление 0 bar</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Привод форточек через PCA9685; док. §1.5/§2.4; MG996R 180° с металлическими шестернями</t>
+          <t>Привод форточек через PCA9685; док. 03 §1.5 / 04 §2.4; MG996R 180° с металлическими шестернями</t>
         </is>
       </c>
     </row>
@@ -1950,84 +1950,131 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
+          <t>Drip tape 16 mm emitter spacing 20 cm roll 100 m</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="2" t="n">
+        <v>590</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>910</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Lemana PRO</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>590</v>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>https://lemanapro.ru/catalog/search?text=капельная+лента+16+мм+20+см+100</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Капельный полив после YF-S201; док. 03 §2.6.4; Neo-Drip или аналог; + штуцер 1/2→16 мм и фильтр</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Монтаж и запас</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E35" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F35" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Chipdip + Ozon</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="n">
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J34" s="3" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>https://www.chipdip.ru/search?searchtext=кабельные+стяжки+наконечник</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Док. §1.6 сбалансированная строка бюджета (~10% запас); уменьшено после экономии на компонентах</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n"/>
-      <c r="K35" s="2" t="n"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Док. 02 §1.6 сбалансированная строка бюджета (~10% запас); уменьшено после экономии на компонентах</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>ИТОГО (к заказу, qty &gt; 0)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="n">
-        <v>56800</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>13469</v>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="n">
-        <v>43331</v>
-      </c>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="n">
+        <v>58300</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>14379</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>43921</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Без уже имеющегося сетевого оборудования (qty 0); цены проверены июнь 2026</t>
         </is>
@@ -2068,6 +2115,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2101,7 +2149,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>docs/smart-greenhouse-design.md (разделы 1.1–1.6)</t>
+          <t>docs/02-components-and-server.md, 03-greenhouse-installation.md, 04-esp32-and-cabinet.md (§1.1–1.6); index: smart-greenhouse-design.md</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2197,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>56,800 RUB</t>
+          <t>58,300 RUB</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2209,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>43,331 RUB</t>
+          <t>43,921 RUB</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2221,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13,469 RUB</t>
+          <t>14,379 RUB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document optional computer vision and align install ops with real greenhouse conditions.
Add CV design (Yandex cloud, Radxa edge SBC, Hugging Face models), П-layout cameras with photoperiod capture, and HA/script stubs coupled to vent and irrigation. Clarify outdoor entrance cabinet, 70–95% RH, condensation, and winter demount across docs and helpers; refresh BOM via generate_bom.py.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/smart-greenhouse-bom.xlsx
+++ b/docs/smart-greenhouse-bom.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Полевой щит у теплицы; док. 04 §1.3; DKC R5ST0342 с монтажной платой</t>
+          <t>Полевой щит снаружи у входа теплицы (не внутри RH 70–95%); док. 04 §1.3 / 03 §0; DKC R5ST0342 с монтажной платой</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Линии датчиков внутрь теплицы; док. 04 §1.3/04 §2.5; Extralink EX.32341 или аналог DKC outdoor FTP</t>
+          <t>Из щита снаружи в теплицу (датчики, GPIO); doc. 04 §1.3/04 §2.5; Extralink EX.32341 или аналог DKC outdoor FTP</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Антиконденсат в корпусе; док. 04 §1.3/01 §5.1; вентиляционный винт IP67 (аналог Gore vent)</t>
+          <t>Антиконденсат: щит снаружи у влажного входа; док. 04 §1.3/01 §5.1; вентиляционный винт IP67 (аналог Gore vent)</t>
         </is>
       </c>
     </row>
@@ -1992,89 +1992,371 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>PoE IP camera 5 MP IP66/IP67 (Reolink RLC-410 or analog)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>7500</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ozon.ru/search/?text=Reolink+RLC-410+PoE</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>CV‑1 коридор у входа + CV‑2 излом П; RTSP; док. 05 §3 / 03 §1.4.2; не в базовом BOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor Cat6 to greenhouse (cameras, if no spare)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Chipdip</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chipdip.ru/search?searchtext=кабель+Cat6+наружный</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>30–40 m к PoE‑коммутатору; shared conduit с ESP32 или отдельная трасса; док. 05 §3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>GORE vent + drip loop kit for cameras (×2)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+камера</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Антиконденсат на корпусе; doc. 05 §3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Radxa ZERO 3W 1GB RAM / 8GB eMMC (edge CV host)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3790</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>410</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>onpad.ru</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>3790</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>https://onpad.ru/catalog/cubie/radxa/rock/radxa_zero_series/3542.html</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>greenhouse-cv-edge · .13 · RTSP + ONNX; doc. 05 §3.4 / 04 §1.4; не ESP32</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>USB-C buck 5V 3A (edge SBC power from LRS-50-5)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Chipdip</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chipdip.ru/search?searchtext=USB-C+5V+3A+buck</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Питание edge SBC от щита; doc. 04 §2.5 / 05 §3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>microSD 32GB (edge SBC backup, optional with eMMC)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ozon.ru/search/?text=microSD+32GB+Class10</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Резервная загрузка Radxa; doc. 05 §3.4 — опционально при 8GB eMMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>Монтаж и запас</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
         </is>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D41" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E41" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F41" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Chipdip + Ozon</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="n">
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J35" s="3" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>https://www.chipdip.ru/search?searchtext=кабельные+стяжки+наконечник</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Док. 02 §1.6 сбалансированная строка бюджета (~10% запас); уменьшено после экономии на компонентах</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Док. 02 §1.6; incl. silica gel 50–100 g для щита снаружи (doc. 04 §1.3); ~10% запас</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>ИТОГО (к заказу, qty &gt; 0)</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="n">
-        <v>58300</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>14379</v>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="n">
-        <v>43921</v>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="n">
+        <v>86600</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>19439</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>67161</v>
+      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Без уже имеющегося сетевого оборудования (qty 0); цены проверены июнь 2026</t>
         </is>
@@ -2116,6 +2398,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2149,7 +2437,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>docs/02-components-and-server.md, 03-greenhouse-installation.md, 04-esp32-and-cabinet.md (§1.1–1.6); index: smart-greenhouse-design.md</t>
+          <t>docs/02-components-and-server.md, 03-greenhouse-installation.md, 04-esp32-and-cabinet.md (§1.1–1.6), 05-computer-vision.md (optional CV); index: smart-greenhouse-design.md</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2485,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>58,300 RUB</t>
+          <t>86,600 RUB</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2497,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>43,921 RUB</t>
+          <t>67,161 RUB</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2509,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14,379 RUB</t>
+          <t>19,439 RUB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add tank level calibration and uv script config
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/smart-greenhouse-bom.xlsx
+++ b/docs/smart-greenhouse-bom.xlsx
@@ -1584,7 +1584,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Capacitor 100 nF (float switch debounce)</t>
+          <t>Capacitor 100 nF (level contact debounce, optional)</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; опциональный debounce поплавка; док. 01 §5.2 — кол‑во 0 к заказу</t>
+          <t>Уже есть; опциональный аппаратный debounce контактного уровня; док. 01 §5.2 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -1762,20 +1762,20 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Float switch level sensor (12–24 V NO/NC)</t>
+          <t>Stainless tank level contacts kit (3 bolts + ring terminals)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>350</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -1788,16 +1788,16 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=поплавковый+датчик+уровня+воды+12V</t>
+          <t>https://www.ozon.ru/search/?text=болт+нержавеющий+M4+клемма+кольцевая</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Верхний уровень бака; док. 03 §1.4 / 04 §2.2; бытовой поплавок (не промышленный ПДУ)</t>
+          <t>Три контакта в баке: верхний, средний, нижний общий; док. 03 §1.4 / 04 §2.2</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
         <v>86600</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>19439</v>
+        <v>19519</v>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="I43" s="4" t="n">
-        <v>67161</v>
+        <v>67081</v>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>67,161 RUB</t>
+          <t>67,081 RUB</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>19,439 RUB</t>
+          <t>19,519 RUB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add soil moisture sensor calibration
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/smart-greenhouse-bom.xlsx
+++ b/docs/smart-greenhouse-bom.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1551,19 +1551,25 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Chipdip</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>RUB</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
@@ -1572,7 +1578,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; подтяжки DS18B20 + I2C; док. 04 §2.1 — кол‑во 0 к заказу</t>
+          <t>Подтяжки DS18B20 + I2C ADS1115 на ESP32 №1 (GPIO21/22); doc. 04 §2.1</t>
         </is>
       </c>
     </row>
@@ -1762,24 +1768,24 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Stainless tank level contacts kit (3 bolts + ring terminals)</t>
+          <t>Sealed capacitive soil moisture probe analog IP68 (Vegetronix VH400 class)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>350</v>
+        <v>1200</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>150</v>
+        <v>1800</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Ozon / AliExpress</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1788,16 +1794,16 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>200</v>
+        <v>5400</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=болт+нержавеющий+M4+клемма+кольцевая</t>
+          <t>https://www.ozon.ru/search/?text=Vegetronix+VH400+soil+moisture</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Три контакта в баке: верхний, средний, нижний общий; док. 03 §1.4 / 04 §2.2</t>
+          <t>П‑layout: 3 зонда на плечо L/R; корень 10–15 cm; сезон в мокрой почве; не резистивные модули; doc. 03 §1.4.3 / 04 §2.2</t>
         </is>
       </c>
     </row>
@@ -1809,20 +1815,20 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>YF-S201 water flow sensor 1/2 inch</t>
+          <t>ADS1115 16-bit I2C ADC module</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>248</v>
+        <v>220</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>450</v>
+        <v>280</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>404</v>
+        <v>120</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -1835,45 +1841,45 @@
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>496</v>
+        <v>440</v>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/product/datchik-rashoda-vody-yf-s201</t>
+          <t>https://www.youbot.ru/search?q=ADS1115</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Учёт полива и наполнения бака; док. 03 §1.4</t>
+          <t>ESP32 watering: ADDR 0x48 + 0x49; 6 analog soil channels; GPIO21/22; doc. 04 §2.2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Исполнительные устройства</t>
+          <t>Датчики</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Solenoid valve NC 12 V 1/2 inch brass</t>
+          <t>Stainless tank level contacts kit (3 bolts + ring terminals)</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>617</v>
+        <v>200</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>900</v>
+        <v>350</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>566</v>
+        <v>150</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>AliExpress (alishops.ru)</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1882,41 +1888,41 @@
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>1234</v>
+        <v>200</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>https://alishops.ru/product-ebowan-g1-2-latunniy-elektricheskiy-elektromagnitniy-klapan-n-c-12v-24v-220v-g3-4-vodniy-vozdushniy-vpusknoy-pereklyuchatel-potoka-dlya-solnechnogo-vodonagrevatelya-klapan/32917349764</t>
+          <t>https://www.ozon.ru/search/?text=болт+нержавеющий+M4+клемма+кольцевая</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Полив + наполнение бака; fail-safe NC; док. 03 §1.5; латунь 12 V DC прямого действия; реселлер AliExpress — проверить NC и мин. давление 0 bar</t>
+          <t>Три контакта в баке: верхний, средний, нижний общий; док. 03 §1.4 / 04 §2.2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Исполнительные устройства</t>
+          <t>Датчики</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>MG996R servo (metal gears)</t>
+          <t>YF-S201 water flow sensor 1/2 inch</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>320</v>
+        <v>248</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>450</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>260</v>
+        <v>404</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -1929,45 +1935,45 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>640</v>
+        <v>496</v>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/product/servoprivod-mg996r-180-gradusov-metall</t>
+          <t>https://www.youbot.ru/product/datchik-rashoda-vody-yf-s201</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Привод форточек через PCA9685; док. 03 §1.5 / 04 §2.4; MG996R 180° с металлическими шестернями</t>
+          <t>Учёт полива и наполнения бака; док. 03 §1.4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Монтаж и запас</t>
+          <t>Исполнительные устройства</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Drip tape 16 mm emitter spacing 20 cm roll 100 m</t>
+          <t>Solenoid valve NC 12 V 1/2 inch brass</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>590</v>
+        <v>617</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>910</v>
+        <v>566</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Lemana PRO</t>
+          <t>AliExpress (alishops.ru)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1976,45 +1982,45 @@
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>590</v>
+        <v>1234</v>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalog/search?text=капельная+лента+16+мм+20+см+100</t>
+          <t>https://alishops.ru/product-ebowan-g1-2-latunniy-elektricheskiy-elektromagnitniy-klapan-n-c-12v-24v-220v-g3-4-vodniy-vozdushniy-vpusknoy-pereklyuchatel-potoka-dlya-solnechnogo-vodonagrevatelya-klapan/32917349764</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Капельный полив после YF-S201; док. 03 §2.6.4; Neo-Drip или аналог; + штуцер 1/2→16 мм и фильтр</t>
+          <t>Полив + наполнение бака; fail-safe NC; док. 03 §1.5; латунь 12 V DC прямого действия; реселлер AliExpress — проверить NC и мин. давление 0 bar</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Computer vision (optional)</t>
+          <t>Исполнительные устройства</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>PoE IP camera 5 MP IP66/IP67 (Reolink RLC-410 or analog)</t>
+          <t>MG996R servo (metal gears)</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>7500</v>
+        <v>320</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>9000</v>
+        <v>450</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>3000</v>
+        <v>260</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Youbot</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2023,45 +2029,45 @@
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>15000</v>
+        <v>640</v>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Reolink+RLC-410+PoE</t>
+          <t>https://www.youbot.ru/product/servoprivod-mg996r-180-gradusov-metall</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>CV‑1 коридор у входа + CV‑2 излом П; RTSP; док. 05 §3 / 03 §1.4.2; не в базовом BOM</t>
+          <t>Привод форточек через PCA9685; док. 03 §1.5 / 04 §2.4; MG996R 180° с металлическими шестернями</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Computer vision (optional)</t>
+          <t>Монтаж и запас</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Outdoor Cat6 to greenhouse (cameras, if no spare)</t>
+          <t>Drip tape 16 mm emitter spacing 20 cm roll 100 m</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>2500</v>
+        <v>590</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>3200</v>
+        <v>1500</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>700</v>
+        <v>910</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Chipdip</t>
+          <t>Lemana PRO</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2070,16 +2076,16 @@
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>2500</v>
+        <v>590</v>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=кабель+Cat6+наружный</t>
+          <t>https://lemanapro.ru/catalog/search?text=капельная+лента+16+мм+20+см+100</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>30–40 m к PoE‑коммутатору; shared conduit с ESP32 или отдельная трасса; док. 05 §3.4</t>
+          <t>Капельный полив после YF-S201; док. 03 §2.6.4; Neo-Drip или аналог; + штуцер 1/2→16 мм и фильтр</t>
         </is>
       </c>
     </row>
@@ -2091,20 +2097,20 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>GORE vent + drip loop kit for cameras (×2)</t>
+          <t>PoE IP camera 5 MP IP66/IP67 (Reolink RLC-410 or analog)</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1000</v>
+        <v>7500</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1600</v>
+        <v>9000</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>600</v>
+        <v>3000</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -2117,16 +2123,16 @@
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>1000</v>
+        <v>15000</v>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+камера</t>
+          <t>https://www.ozon.ru/search/?text=Reolink+RLC-410+PoE</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Антиконденсат на корпусе; doc. 05 §3.3</t>
+          <t>CV‑1 коридор у входа + CV‑2 излом П; RTSP; док. 05 §3 / 03 §1.4.2; не в базовом BOM</t>
         </is>
       </c>
     </row>
@@ -2138,24 +2144,24 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Radxa ZERO 3W 1GB RAM / 8GB eMMC (edge CV host)</t>
+          <t>Outdoor Cat6 to greenhouse (cameras, if no spare)</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>3790</v>
+        <v>2500</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>4200</v>
+        <v>3200</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>410</v>
+        <v>700</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>onpad.ru</t>
+          <t>Chipdip</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2164,16 +2170,16 @@
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>3790</v>
+        <v>2500</v>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>https://onpad.ru/catalog/cubie/radxa/rock/radxa_zero_series/3542.html</t>
+          <t>https://www.chipdip.ru/search?searchtext=кабель+Cat6+наружный</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>greenhouse-cv-edge · .13 · RTSP + ONNX pre-filter · local post to Pi; no WAN; doc. 05 §3.4 / 04 §1.4</t>
+          <t>30–40 m к PoE‑коммутатору; shared conduit с ESP32 или отдельная трасса; док. 05 §3.4</t>
         </is>
       </c>
     </row>
@@ -2185,24 +2191,24 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>USB-C buck 5V 3A (edge SBC power from LRS-50-5)</t>
+          <t>GORE vent + drip loop kit for cameras (×2)</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>450</v>
+        <v>1000</v>
       </c>
       <c r="E39" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F39" s="2" t="n">
         <v>600</v>
       </c>
-      <c r="F39" s="2" t="n">
-        <v>150</v>
-      </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Chipdip</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2211,16 +2217,16 @@
         </is>
       </c>
       <c r="I39" s="2" t="n">
-        <v>450</v>
+        <v>1000</v>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=USB-C+5V+3A+buck</t>
+          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+камера</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Питание edge SBC от щита; doc. 04 §2.5 / 05 §3.4</t>
+          <t>Антиконденсат на корпусе; doc. 05 §3.3</t>
         </is>
       </c>
     </row>
@@ -2232,24 +2238,24 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>microSD 32GB (edge SBC backup, optional with eMMC)</t>
+          <t>Radxa ZERO 3W 1GB RAM / 8GB eMMC (edge CV host)</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>500</v>
+        <v>3790</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>700</v>
+        <v>4200</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>200</v>
+        <v>410</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>onpad.ru</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2258,105 +2264,199 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>500</v>
+        <v>3790</v>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=microSD+32GB+Class10</t>
+          <t>https://onpad.ru/catalog/cubie/radxa/rock/radxa_zero_series/3542.html</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Резервная загрузка Radxa; doc. 05 §3.4 — опционально при 8GB eMMC</t>
+          <t>greenhouse-cv-edge · .13 · RTSP + ONNX pre-filter · local post to Pi; no WAN; doc. 05 §3.4 / 04 §1.4</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Монтаж и запас</t>
+          <t>Computer vision (optional)</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
+          <t>USB-C buck 5V 3A (edge SBC power from LRS-50-5)</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D41" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Chipdip</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chipdip.ru/search?searchtext=USB-C+5V+3A+buck</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Питание edge SBC от щита; doc. 04 §2.5 / 05 §3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>microSD 32GB (edge SBC backup, optional with eMMC)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ozon.ru/search/?text=microSD+32GB+Class10</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Резервная загрузка Radxa; doc. 05 §3.4 — опционально при 8GB eMMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Монтаж и запас</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="E41" s="2" t="n">
+      <c r="E43" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="F43" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Chipdip + Ozon</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="n">
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J41" s="3" t="inlineStr">
+      <c r="J43" s="3" t="inlineStr">
         <is>
           <t>https://www.chipdip.ru/search?searchtext=кабельные+стяжки+наконечник</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Док. 02 §1.6; incl. silica gel 50–100 g для щита снаружи (doc. 04 §1.3); ~10% запас</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
-      <c r="J42" s="2" t="n"/>
-      <c r="K42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-      <c r="B43" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
+      <c r="K44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>ИТОГО (к заказу, qty &gt; 0)</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr"/>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="n">
-        <v>86600</v>
-      </c>
-      <c r="F43" s="4" t="n">
-        <v>19519</v>
-      </c>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="n">
-        <v>67081</v>
-      </c>
-      <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="n">
+        <v>94360</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>21429</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>72931</v>
+      </c>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Без уже имеющегося сетевого оборудования (qty 0); цены проверены июнь 2026</t>
         </is>
@@ -2404,6 +2504,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2485,7 +2587,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>86,600 RUB</t>
+          <t>94,360 RUB</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2599,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>67,081 RUB</t>
+          <t>72,931 RUB</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2611,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>19,519 RUB</t>
+          <t>21,429 RUB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update greenhouse docs for actuator and soil sensor guidance
</commit_message>
<xml_diff>
--- a/docs/smart-greenhouse-bom.xlsx
+++ b/docs/smart-greenhouse-bom.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Драйвер MG996R на greenhouse-climate; док. 04 §1.3/04 §2.4</t>
+          <t>Драйвер текущего MG996R/servo-варианта на greenhouse-climate; для линейных актуаторов не нужен; док. 04 §1.3/04 §2.4</t>
         </is>
       </c>
     </row>
@@ -1218,24 +1218,24 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Enclosure DKC R5ST0342 IP65 300×400×200 mm (metal)</t>
+          <t>Fuse + TVS protection kit for 12 V loads</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>4458</v>
+        <v>800</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>5500</v>
+        <v>1200</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1042</v>
+        <v>400</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Electroprice</t>
+          <t>Chipdip</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1244,16 +1244,16 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>4458</v>
+        <v>800</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>https://electroprice.ru/product/shkaf-st-s-montazh--platoy-300h400h200mm-ot-ip65-do-ip66-ik10-dkc-r5st0342/117349</t>
+          <t>https://www.chipdip.ru/search?searchtext=предохранитель+TVS+12V</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Полевой щит снаружи у входа теплицы (не внутри RH 70–95%); док. 04 §1.3 / 03 §0; DKC R5ST0342 с монтажной платой</t>
+          <t>Предохранитель на силовую линию, TVS/защита моторов и клеммы; док. 04 §2.1; не экономить на силовой части</t>
         </is>
       </c>
     </row>
@@ -1265,24 +1265,24 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>WAGO 221 terminals + cable glands PG7/PG9/PG11 + DIN rail kit</t>
+          <t>Enclosure DKC R5ST0342 IP65 300×400×200 mm (metal)</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1800</v>
+        <v>4458</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2500</v>
+        <v>5500</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>700</v>
+        <v>1042</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Chipdip + IEK</t>
+          <t>Electroprice</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1291,16 +1291,16 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1800</v>
+        <v>4458</v>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=WAGO+221+набор</t>
+          <t>https://electroprice.ru/product/shkaf-st-s-montazh--platoy-300h400h200mm-ot-ip65-do-ip66-ik10-dkc-r5st0342/117349</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>1 комплект; WAGO 221 + сальники DKC PG + DIN‑рейка; док. 04 §1.3; оценка набора</t>
+          <t>Полевой щит снаружи у входа теплицы (не внутри RH 70–95%); док. 04 §1.3 / 03 §0; DKC R5ST0342 с монтажной платой</t>
         </is>
       </c>
     </row>
@@ -1312,24 +1312,24 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>FTP Cat5e outdoor cable (50 m roll)</t>
+          <t>WAGO 221 terminals + cable glands PG7/PG9/PG11 + DIN rail kit</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2800</v>
+        <v>2500</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Chipdip + IEK</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1338,16 +1338,16 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Extralink+Cat5e+FTP+outdoor+50m</t>
+          <t>https://www.chipdip.ru/search?searchtext=WAGO+221+набор</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Из щита снаружи в теплицу (датчики, GPIO); doc. 04 §1.3/04 §2.5; Extralink EX.32341 или аналог DKC outdoor FTP</t>
+          <t>1 комплект; WAGO 221 + сальники DKC PG + DIN‑рейка; док. 04 §1.3; оценка набора</t>
         </is>
       </c>
     </row>
@@ -1359,17 +1359,17 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Mini UPS 12 V DC 3 A (optional)</t>
+          <t>FTP Cat5e outdoor cable (50 m roll)</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2400</v>
+        <v>2200</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>3000</v>
+        <v>2800</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>600</v>
@@ -1385,16 +1385,16 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>2400</v>
+        <v>2200</v>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=mini+UPS+12V+DC+3A+WGP</t>
+          <t>https://www.ozon.ru/search/?text=Extralink+Cat5e+FTP+outdoor+50m</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Опционально; удерживает клапаны в безопасном состоянии при отключении питания; док. 04 §1.3/01 §6.4; класс WGP V1203</t>
+          <t>Из щита снаружи в теплицу (датчики, GPIO); doc. 04 §1.3/04 §2.5; Extralink EX.32341 или аналог DKC outdoor FTP</t>
         </is>
       </c>
     </row>
@@ -1406,20 +1406,20 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Gore vent IP67 (pressure equalization)</t>
+          <t>Mini UPS 12 V DC 3 A (optional)</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>450</v>
+        <v>2400</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>700</v>
+        <v>3000</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1432,16 +1432,16 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>450</v>
+        <v>2400</v>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+электрощит</t>
+          <t>https://www.ozon.ru/search/?text=mini+UPS+12V+DC+3A+WGP</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Антиконденсат: щит снаружи у влажного входа; док. 04 §1.3/01 §5.1; вентиляционный винт IP67 (аналог Gore vent)</t>
+          <t>Опционально; удерживает клапаны в безопасном состоянии при отключении питания; док. 04 §1.3/01 §6.4; класс WGP V1203</t>
         </is>
       </c>
     </row>
@@ -1453,24 +1453,24 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Circuit breaker 10 A (220 V AC input)</t>
+          <t>Gore vent IP67 (pressure equalization)</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>220</v>
+        <v>450</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Chipdip</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1479,16 +1479,16 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>220</v>
+        <v>450</v>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=автомат+10А+IEK</t>
+          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+электрощит</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Оценка; док. 04 §2.5/01 §6.4; IEK/DEK 1P 10 A</t>
+          <t>Антиконденсат: щит снаружи у влажного входа; док. 04 §1.3/01 §5.1; вентиляционный винт IP67 (аналог Gore vent)</t>
         </is>
       </c>
     </row>
@@ -1500,20 +1500,20 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>PSU 5 V ≥3 A for servo V+ on PCA9685</t>
+          <t>Circuit breaker 10 A (220 V AC input)</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>550</v>
+        <v>220</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>450</v>
+        <v>180</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -1526,16 +1526,16 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>550</v>
+        <v>220</v>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=DL-15W-V5-EXC</t>
+          <t>https://www.chipdip.ru/search?searchtext=автомат+10А+IEK</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Отдельно от LRS-50-5; док. 04 §2.4/01 §5.2; закрытый БП DONE 5 V 3 A 15 W</t>
+          <t>Оценка; док. 04 §2.5/01 §6.4; IEK/DEK 1P 10 A</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,21 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Resistor 4.7 kΩ (I2C / OneWire pull-up)</t>
+          <t>PSU 5 V ≥3 A for servo V+ on PCA9685</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+        <v>550</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>450</v>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Chipdip</t>
@@ -1569,16 +1573,16 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>10</v>
+        <v>550</v>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=резистор+4.7+кОм</t>
+          <t>https://www.chipdip.ru/search?searchtext=DL-15W-V5-EXC</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Подтяжки DS18B20 + I2C ADS1115 на ESP32 №1 (GPIO21/22); doc. 04 §2.1</t>
+          <t>Только если оставлять MG996R; отдельно от LRS-50-5; док. 04 §2.4/01 §5.2; закрытый БП DONE 5 V 3 A 15 W</t>
         </is>
       </c>
     </row>
@@ -1590,79 +1594,75 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Capacitor 100 nF (level contact debounce, optional)</t>
+          <t>Resistor 4.7 kΩ (I2C / OneWire pull-up)</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Chipdip</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>RUB</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=конденсатор+100нФ</t>
+          <t>https://www.chipdip.ru/search?searchtext=резистор+4.7+кОм</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Уже есть; опциональный аппаратный debounce контактного уровня; док. 01 §5.2 — кол‑во 0 к заказу</t>
+          <t>Подтяжки DS18B20 + I2C ADS1115 на ESP32 №1 (GPIO21/22); doc. 04 §2.1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Датчики</t>
+          <t>Щит IP65 у теплицы</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>SHT31 temperature/humidity module (GY-SHT31-D)</t>
+          <t>Capacitor 100 nF (level contact debounce, optional)</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>295</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>350</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>165</v>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Youbot</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>RUB</t>
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>885</v>
+        <v>0</v>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/product/tsifrovoy-datchik-temperatury-i-vlazhnosti-gy-sht31d</t>
+          <t>https://www.chipdip.ru/search?searchtext=конденсатор+100нФ</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Вход низ, центр наверху, противоположная сторона; I2C 0x44/0x45; док. 03 §1.4.1 / 04 §2.3</t>
+          <t>Уже есть; опциональный аппаратный debounce контактного уровня; док. 01 §5.2 — кол‑во 0 к заказу</t>
         </is>
       </c>
     </row>
@@ -1674,24 +1674,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>BH1750 light sensor module (GY-302)</t>
+          <t>AHT20/AHT21 temperature/humidity module (budget option)</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>119</v>
+        <v>180</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>162</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Youbot</t>
+          <t>Ozon / AliExpress</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1700,16 +1698,16 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>238</v>
+        <v>0</v>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/product/gy-302-bh1750-datchik-sveta</t>
+          <t>https://www.ozon.ru/search/?text=AHT20+I2C+датчик+влажности</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Потолок + уровень растений; док. 03 §1.4</t>
+          <t>Бюджетная альтернатива SHT31; ставить в вентилируемый экран, не в прямой конденсат; док. 03 §1.4</t>
         </is>
       </c>
     </row>
@@ -1721,24 +1719,24 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>DS18B20 waterproof temperature probe (1 m)</t>
+          <t>SHT31 temperature/humidity module (GY-SHT31-D)</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>190</v>
+        <v>295</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>20</v>
+        <v>165</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>YourDuino</t>
+          <t>Youbot</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1747,16 +1745,16 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>380</v>
+        <v>885</v>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>https://www.yourduino.ru/product/vodonepronitsaemyy-temperaturnyy-datchik-zond-ds18b20</t>
+          <t>https://www.youbot.ru/product/tsifrovoy-datchik-temperatury-i-vlazhnosti-gy-sht31d</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Бак + линия полива; OneWire; док. 03 §1.4 / 04 §2.2</t>
+          <t>Вход низ, центр наверху, противоположная сторона; I2C 0x44/0x45; док. 03 §1.4.1 / 04 §2.3</t>
         </is>
       </c>
     </row>
@@ -1768,24 +1766,24 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Sealed capacitive soil moisture probe analog IP68 (Vegetronix VH400 class)</t>
+          <t>BH1750 light sensor module (GY-302)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>900</v>
+        <v>119</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>1200</v>
+        <v>200</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1800</v>
+        <v>162</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Ozon / AliExpress</t>
+          <t>Youbot</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1794,16 +1792,16 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>5400</v>
+        <v>238</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Vegetronix+VH400+soil+moisture</t>
+          <t>https://www.youbot.ru/product/gy-302-bh1750-datchik-sveta</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>П‑layout: 3 зонда на плечо L/R; корень 10–15 cm; сезон в мокрой почве; не резистивные модули; doc. 03 §1.4.3 / 04 §2.2</t>
+          <t>Потолок + уровень растений; док. 03 §1.4</t>
         </is>
       </c>
     </row>
@@ -1815,24 +1813,24 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>ADS1115 16-bit I2C ADC module</t>
+          <t>DS18B20 waterproof temperature probe (1 m)</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Youbot</t>
+          <t>YourDuino</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1841,16 +1839,16 @@
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>440</v>
+        <v>380</v>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/search?q=ADS1115</t>
+          <t>https://www.yourduino.ru/product/vodonepronitsaemyy-temperaturnyy-datchik-zond-ds18b20</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>ESP32 watering: ADDR 0x48 + 0x49; 6 analog soil channels; GPIO21/22; doc. 04 §2.2</t>
+          <t>Бак + линия полива; OneWire; док. 03 §1.4 / 04 §2.2</t>
         </is>
       </c>
     </row>
@@ -1862,24 +1860,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Stainless tank level contacts kit (3 bolts + ring terminals)</t>
+          <t>Capacitive Soil Moisture Sensor v1.2/v2.0 (budget + spares)</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>350</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>150</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Ozon / AliExpress</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1888,16 +1884,16 @@
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=болт+нержавеющий+M4+клемма+кольцевая</t>
+          <t>https://www.ozon.ru/search/?text=Capacitive+Soil+Moisture+Sensor+v1.2</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Три контакта в баке: верхний, средний, нижний общий; док. 03 §1.4 / 04 §2.2</t>
+          <t>Бюджетная замена VH400: покупать 6+2, герметизировать верх платы, калибровать каждый зонд; не резистивные YL-69/FC-28; док. 03 §1.4.3</t>
         </is>
       </c>
     </row>
@@ -1909,24 +1905,24 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>YF-S201 water flow sensor 1/2 inch</t>
+          <t>Sealed capacitive soil moisture probe analog IP68 (Vegetronix VH400 class)</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>248</v>
+        <v>900</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>450</v>
+        <v>1200</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>404</v>
+        <v>1800</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Youbot</t>
+          <t>Ozon / AliExpress</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1935,45 +1931,45 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>496</v>
+        <v>5400</v>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/product/datchik-rashoda-vody-yf-s201</t>
+          <t>https://www.ozon.ru/search/?text=Vegetronix+VH400+soil+moisture</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Учёт полива и наполнения бака; док. 03 §1.4</t>
+          <t>П‑layout: 3 зонда на плечо L/R; корень 10–15 cm; сезон в мокрой почве; не резистивные модули; doc. 03 §1.4.3 / 04 §2.2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Исполнительные устройства</t>
+          <t>Датчики</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Solenoid valve NC 12 V 1/2 inch brass</t>
+          <t>ADS1115 16-bit I2C ADC module</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>617</v>
+        <v>220</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>900</v>
+        <v>280</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>566</v>
+        <v>120</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>AliExpress (alishops.ru)</t>
+          <t>Youbot</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1982,45 +1978,45 @@
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>1234</v>
+        <v>440</v>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>https://alishops.ru/product-ebowan-g1-2-latunniy-elektricheskiy-elektromagnitniy-klapan-n-c-12v-24v-220v-g3-4-vodniy-vozdushniy-vpusknoy-pereklyuchatel-potoka-dlya-solnechnogo-vodonagrevatelya-klapan/32917349764</t>
+          <t>https://www.youbot.ru/search?q=ADS1115</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Полив + наполнение бака; fail-safe NC; док. 03 §1.5; латунь 12 V DC прямого действия; реселлер AliExpress — проверить NC и мин. давление 0 bar</t>
+          <t>ESP32 watering: ADDR 0x48 + 0x49; 6 analog soil channels; GPIO21/22; doc. 04 §2.2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Исполнительные устройства</t>
+          <t>Датчики</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>MG996R servo (metal gears)</t>
+          <t>Stainless tank level contacts kit (3 bolts + ring terminals)</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>260</v>
+        <v>150</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Youbot</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2029,45 +2025,45 @@
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>https://www.youbot.ru/product/servoprivod-mg996r-180-gradusov-metall</t>
+          <t>https://www.ozon.ru/search/?text=болт+нержавеющий+M4+клемма+кольцевая</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Привод форточек через PCA9685; док. 03 §1.5 / 04 §2.4; MG996R 180° с металлическими шестернями</t>
+          <t>Три контакта в баке: верхний, средний, нижний общий; док. 03 §1.4 / 04 §2.2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Монтаж и запас</t>
+          <t>Датчики</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Drip tape 16 mm emitter spacing 20 cm roll 100 m</t>
+          <t>YF-S201 water flow sensor 1/2 inch</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>590</v>
+        <v>248</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1500</v>
+        <v>450</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>910</v>
+        <v>404</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Lemana PRO</t>
+          <t>Youbot</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2076,45 +2072,45 @@
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>590</v>
+        <v>496</v>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalog/search?text=капельная+лента+16+мм+20+см+100</t>
+          <t>https://www.youbot.ru/product/datchik-rashoda-vody-yf-s201</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Капельный полив после YF-S201; док. 03 §2.6.4; Neo-Drip или аналог; + штуцер 1/2→16 мм и фильтр</t>
+          <t>Учёт полива и наполнения бака; док. 03 §1.4</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Computer vision (optional)</t>
+          <t>Исполнительные устройства</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>PoE IP camera 5 MP IP66/IP67 (Reolink RLC-410 or analog)</t>
+          <t>Solenoid valve NC 12 V 1/2 inch brass</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>7500</v>
+        <v>617</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>9000</v>
+        <v>900</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>3000</v>
+        <v>566</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>AliExpress (alishops.ru)</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2123,45 +2119,45 @@
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>15000</v>
+        <v>1234</v>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Reolink+RLC-410+PoE</t>
+          <t>https://alishops.ru/product-ebowan-g1-2-latunniy-elektricheskiy-elektromagnitniy-klapan-n-c-12v-24v-220v-g3-4-vodniy-vozdushniy-vpusknoy-pereklyuchatel-potoka-dlya-solnechnogo-vodonagrevatelya-klapan/32917349764</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>CV‑1 коридор у входа + CV‑2 излом П; RTSP; док. 05 §3 / 03 §1.4.2; не в базовом BOM</t>
+          <t>Полив + наполнение бака; fail-safe NC; док. 03 §1.5; латунь 12 V DC прямого действия; реселлер AliExpress — проверить NC и мин. давление 0 bar</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Computer vision (optional)</t>
+          <t>Исполнительные устройства</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Outdoor Cat6 to greenhouse (cameras, if no spare)</t>
+          <t>Linear actuator 12 V with limit switches (IP54/IP65)</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="2" t="n">
         <v>2500</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>3200</v>
+        <v>3500</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>700</v>
+        <v>2000</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Chipdip</t>
+          <t>Ozon / AliExpress</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2170,45 +2166,45 @@
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=кабель+Cat6+наружный</t>
+          <t>https://www.ozon.ru/search/?text=линейный+актуатор+12V+100mm+концевики+IP65</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>30–40 m к PoE‑коммутатору; shared conduit с ESP32 или отдельная трасса; док. 05 §3.4</t>
+          <t>Рекомендуемый привод форточек для реальной эксплуатации; нужен H-bridge/реле реверса и обновление ESPHome; док. 03 §1.5 / 04 §2.4</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Computer vision (optional)</t>
+          <t>Исполнительные устройства</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>GORE vent + drip loop kit for cameras (×2)</t>
+          <t>MG996R servo (metal gears, prototype/light vents only)</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>1000</v>
+        <v>320</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1600</v>
+        <v>450</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>600</v>
+        <v>260</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Youbot</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2217,45 +2213,45 @@
         </is>
       </c>
       <c r="I39" s="2" t="n">
-        <v>1000</v>
+        <v>640</v>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+камера</t>
+          <t>https://www.youbot.ru/product/servoprivod-mg996r-180-gradusov-metall</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Антиконденсат на корпусе; doc. 05 §3.3</t>
+          <t>Текущая ESPHome/PCA9685-схема; только для стенда или лёгких створок, не лучший полевой вариант; док. 03 §1.5 / 04 §2.4</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Computer vision (optional)</t>
+          <t>Монтаж и запас</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Radxa ZERO 3W 1GB RAM / 8GB eMMC (edge CV host)</t>
+          <t>Drip tape 16 mm emitter spacing 20 cm roll 100 m</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>3790</v>
+        <v>590</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>4200</v>
+        <v>1500</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>410</v>
+        <v>910</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>onpad.ru</t>
+          <t>Lemana PRO</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2264,16 +2260,16 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>3790</v>
+        <v>590</v>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>https://onpad.ru/catalog/cubie/radxa/rock/radxa_zero_series/3542.html</t>
+          <t>https://lemanapro.ru/catalog/search?text=капельная+лента+16+мм+20+см+100</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>greenhouse-cv-edge · .13 · RTSP + ONNX pre-filter · local post to Pi; no WAN; doc. 05 §3.4 / 04 §1.4</t>
+          <t>Капельный полив после YF-S201; док. 03 §2.6.4; Neo-Drip или аналог; + штуцер 1/2→16 мм и фильтр</t>
         </is>
       </c>
     </row>
@@ -2285,24 +2281,24 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>USB-C buck 5V 3A (edge SBC power from LRS-50-5)</t>
+          <t>PoE IP camera 5 MP IP66/IP67 (Reolink RLC-410 or analog)</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>450</v>
+        <v>7500</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>600</v>
+        <v>9000</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>150</v>
+        <v>3000</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Chipdip</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2311,16 +2307,16 @@
         </is>
       </c>
       <c r="I41" s="2" t="n">
-        <v>450</v>
+        <v>15000</v>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>https://www.chipdip.ru/search?searchtext=USB-C+5V+3A+buck</t>
+          <t>https://www.ozon.ru/search/?text=Reolink+RLC-410+PoE</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Питание edge SBC от щита; doc. 04 §2.5 / 05 §3.4</t>
+          <t>CV‑1 коридор у входа + CV‑2 излом П; RTSP; док. 05 §3 / 03 §1.4.2; не в базовом BOM</t>
         </is>
       </c>
     </row>
@@ -2332,24 +2328,24 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>microSD 32GB (edge SBC backup, optional with eMMC)</t>
+          <t>Outdoor Cat6 to greenhouse (cameras, if no spare)</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="E42" s="2" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F42" s="2" t="n">
         <v>700</v>
       </c>
-      <c r="F42" s="2" t="n">
-        <v>200</v>
-      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Chipdip</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2358,105 +2354,293 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>https://www.ozon.ru/search/?text=microSD+32GB+Class10</t>
+          <t>https://www.chipdip.ru/search?searchtext=кабель+Cat6+наружный</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Резервная загрузка Radxa; doc. 05 §3.4 — опционально при 8GB eMMC</t>
+          <t>30–40 m к PoE‑коммутатору; shared conduit с ESP32 или отдельная трасса; док. 05 §3.4</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Монтаж и запас</t>
+          <t>Computer vision (optional)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
+          <t>GORE vent + drip loop kit for cameras (×2)</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D43" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ozon.ru/search/?text=Gore+vent+IP67+камера</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Антиконденсат на корпусе; doc. 05 §3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Radxa ZERO 3W 1GB RAM / 8GB eMMC (edge CV host)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>3790</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>410</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>onpad.ru</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>3790</v>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>https://onpad.ru/catalog/cubie/radxa/rock/radxa_zero_series/3542.html</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>greenhouse-cv-edge · .13 · RTSP + ONNX pre-filter · local post to Pi; no WAN; doc. 05 §3.4 / 04 §1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>USB-C buck 5V 3A (edge SBC power from LRS-50-5)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Chipdip</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chipdip.ru/search?searchtext=USB-C+5V+3A+buck</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Питание edge SBC от щита; doc. 04 §2.5 / 05 §3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Computer vision (optional)</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>microSD 32GB (edge SBC backup, optional with eMMC)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ozon.ru/search/?text=microSD+32GB+Class10</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Резервная загрузка Radxa; doc. 05 §3.4 — опционально при 8GB eMMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Монтаж и запас</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Cable ties, ferrules, wire, fuses, silica gel, misc.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="E43" s="2" t="n">
+      <c r="E47" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="F47" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Chipdip + Ozon</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="n">
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J43" s="3" t="inlineStr">
+      <c r="J47" s="3" t="inlineStr">
         <is>
           <t>https://www.chipdip.ru/search?searchtext=кабельные+стяжки+наконечник</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Док. 02 §1.6; incl. silica gel 50–100 g для щита снаружи (doc. 04 §1.3); ~10% запас</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
-      <c r="B45" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>ИТОГО (к заказу, qty &gt; 0)</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr"/>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="n">
-        <v>94360</v>
-      </c>
-      <c r="F45" s="4" t="n">
-        <v>21429</v>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="n">
-        <v>72931</v>
-      </c>
-      <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="n">
+        <v>102560</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>23829</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>78731</v>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>Без уже имеющегося сетевого оборудования (qty 0); цены проверены июнь 2026</t>
         </is>
@@ -2506,6 +2690,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2587,7 +2775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>94,360 RUB</t>
+          <t>102,560 RUB</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>72,931 RUB</t>
+          <t>78,731 RUB</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2799,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>21,429 RUB</t>
+          <t>23,829 RUB</t>
         </is>
       </c>
     </row>

</xml_diff>